<commit_message>
fix(catalog): resolve stock display bug, enable editable dropdowns across all fields, and add multi-image upload with Windows path auto-normalization
</commit_message>
<xml_diff>
--- a/Barcode Master.xlsx
+++ b/Barcode Master.xlsx
@@ -995,7 +995,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z1008"/>
+  <dimension ref="A1:Z1014"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1" outlineLevelRow="1"/>
   <cols>
     <col width="9.33203125" customWidth="1" min="1" max="1"/>
@@ -32455,6 +32455,528 @@
       <c r="T1008" t="inlineStr">
         <is>
           <t>PDE26_C1B1F4103313</t>
+        </is>
+      </c>
+    </row>
+    <row r="1009">
+      <c r="A1009" t="n">
+        <v>42</v>
+      </c>
+      <c r="B1009" t="inlineStr">
+        <is>
+          <t>Everyday</t>
+        </is>
+      </c>
+      <c r="C1009" t="inlineStr">
+        <is>
+          <t>DE26011N</t>
+        </is>
+      </c>
+      <c r="D1009" t="inlineStr">
+        <is>
+          <t>Nighty</t>
+        </is>
+      </c>
+      <c r="E1009" t="inlineStr">
+        <is>
+          <t>Short Sleeves</t>
+        </is>
+      </c>
+      <c r="F1009" t="inlineStr">
+        <is>
+          <t>Square Neck</t>
+        </is>
+      </c>
+      <c r="G1009" t="inlineStr">
+        <is>
+          <t>SINGLE DRESS</t>
+        </is>
+      </c>
+      <c r="H1009" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="I1009" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="J1009" t="n">
+        <v>1</v>
+      </c>
+      <c r="K1009" t="inlineStr">
+        <is>
+          <t>Blue</t>
+        </is>
+      </c>
+      <c r="L1009" t="inlineStr">
+        <is>
+          <t>XXL</t>
+        </is>
+      </c>
+      <c r="M1009" t="n">
+        <v>1</v>
+      </c>
+      <c r="N1009" t="inlineStr">
+        <is>
+          <t>DE26011N103613</t>
+        </is>
+      </c>
+      <c r="O1009" t="n">
+        <v>185</v>
+      </c>
+      <c r="P1009" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="Q1009">
+        <f>ROUND($O1009+10+($O1009*0.2)+(($O1009+10+($O1009*0.2))*$P1009)+(($O1009+10+($O1009*0.2)+(($O1009+10+($O1009*0.2))*$P1009))*0.05),0)</f>
+        <v/>
+      </c>
+      <c r="R1009" t="n">
+        <v>449</v>
+      </c>
+      <c r="S1009" t="n">
+        <v>449</v>
+      </c>
+      <c r="T1009" t="inlineStr">
+        <is>
+          <t>PDE26011N103613</t>
+        </is>
+      </c>
+    </row>
+    <row r="1010">
+      <c r="A1010" t="n">
+        <v>50</v>
+      </c>
+      <c r="B1010" t="inlineStr">
+        <is>
+          <t>Everyday</t>
+        </is>
+      </c>
+      <c r="C1010" t="inlineStr">
+        <is>
+          <t>DE26_A6A560</t>
+        </is>
+      </c>
+      <c r="D1010" t="inlineStr">
+        <is>
+          <t>Nighty</t>
+        </is>
+      </c>
+      <c r="E1010" t="inlineStr">
+        <is>
+          <t>Sleeveless</t>
+        </is>
+      </c>
+      <c r="F1010" t="inlineStr">
+        <is>
+          <t>Square Neck</t>
+        </is>
+      </c>
+      <c r="G1010" t="inlineStr">
+        <is>
+          <t>SINGLE DRESS</t>
+        </is>
+      </c>
+      <c r="H1010" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="I1010" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="J1010" t="n">
+        <v>1</v>
+      </c>
+      <c r="K1010" t="inlineStr">
+        <is>
+          <t>Teal</t>
+        </is>
+      </c>
+      <c r="L1010" t="inlineStr">
+        <is>
+          <t>XXL</t>
+        </is>
+      </c>
+      <c r="M1010" t="n">
+        <v>1</v>
+      </c>
+      <c r="N1010" t="inlineStr">
+        <is>
+          <t>DE26_A6A560103313</t>
+        </is>
+      </c>
+      <c r="O1010" t="n">
+        <v>210</v>
+      </c>
+      <c r="P1010" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="Q1010">
+        <f>ROUND($O1010+10+($O1010*0.2)+(($O1010+10+($O1010*0.2))*$P1010)+(($O1010+10+($O1010*0.2)+(($O1010+10+($O1010*0.2))*$P1010))*0.05),0)</f>
+        <v/>
+      </c>
+      <c r="R1010" t="n">
+        <v>499</v>
+      </c>
+      <c r="S1010" t="n">
+        <v>499</v>
+      </c>
+      <c r="T1010" t="inlineStr">
+        <is>
+          <t>PDE26_A6A560103313</t>
+        </is>
+      </c>
+    </row>
+    <row r="1011">
+      <c r="A1011" t="n">
+        <v>51</v>
+      </c>
+      <c r="B1011" t="inlineStr">
+        <is>
+          <t>Everyday</t>
+        </is>
+      </c>
+      <c r="C1011" t="inlineStr">
+        <is>
+          <t>TESTDEL_032328</t>
+        </is>
+      </c>
+      <c r="D1011" t="inlineStr">
+        <is>
+          <t>Women</t>
+        </is>
+      </c>
+      <c r="E1011" t="inlineStr">
+        <is>
+          <t>Nightdress</t>
+        </is>
+      </c>
+      <c r="F1011" t="inlineStr">
+        <is>
+          <t>Maxi</t>
+        </is>
+      </c>
+      <c r="G1011" t="inlineStr">
+        <is>
+          <t>SINGLE DRESS</t>
+        </is>
+      </c>
+      <c r="H1011" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="I1011" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="J1011" t="n">
+        <v>1</v>
+      </c>
+      <c r="K1011" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="L1011" t="inlineStr">
+        <is>
+          <t>XXL</t>
+        </is>
+      </c>
+      <c r="M1011" t="n">
+        <v>1</v>
+      </c>
+      <c r="N1011" t="inlineStr">
+        <is>
+          <t>TESTDEL_032328103813</t>
+        </is>
+      </c>
+      <c r="O1011" t="n">
+        <v>150</v>
+      </c>
+      <c r="P1011" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="Q1011">
+        <f>ROUND($O1011+10+($O1011*0.2)+(($O1011+10+($O1011*0.2))*$P1011)+(($O1011+10+($O1011*0.2)+(($O1011+10+($O1011*0.2))*$P1011))*0.05),0)</f>
+        <v/>
+      </c>
+      <c r="R1011" t="n">
+        <v>499</v>
+      </c>
+      <c r="S1011" t="n">
+        <v>499</v>
+      </c>
+      <c r="T1011" t="inlineStr">
+        <is>
+          <t>PTESTDEL_032328103813</t>
+        </is>
+      </c>
+    </row>
+    <row r="1012">
+      <c r="A1012" t="n">
+        <v>52</v>
+      </c>
+      <c r="B1012" t="inlineStr">
+        <is>
+          <t>Everyday</t>
+        </is>
+      </c>
+      <c r="C1012" t="inlineStr">
+        <is>
+          <t>DE26_C75AC4</t>
+        </is>
+      </c>
+      <c r="D1012" t="inlineStr">
+        <is>
+          <t>Nighty</t>
+        </is>
+      </c>
+      <c r="E1012" t="inlineStr">
+        <is>
+          <t>Sleeveless</t>
+        </is>
+      </c>
+      <c r="F1012" t="inlineStr">
+        <is>
+          <t>Square Neck</t>
+        </is>
+      </c>
+      <c r="G1012" t="inlineStr">
+        <is>
+          <t>SINGLE DRESS</t>
+        </is>
+      </c>
+      <c r="H1012" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="I1012" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="J1012" t="n">
+        <v>1</v>
+      </c>
+      <c r="K1012" t="inlineStr">
+        <is>
+          <t>Teal</t>
+        </is>
+      </c>
+      <c r="L1012" t="inlineStr">
+        <is>
+          <t>XXL</t>
+        </is>
+      </c>
+      <c r="M1012" t="n">
+        <v>1</v>
+      </c>
+      <c r="N1012" t="inlineStr">
+        <is>
+          <t>DE26_C75AC4103313</t>
+        </is>
+      </c>
+      <c r="O1012" t="n">
+        <v>210</v>
+      </c>
+      <c r="P1012" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="Q1012">
+        <f>ROUND($O1012+10+($O1012*0.2)+(($O1012+10+($O1012*0.2))*$P1012)+(($O1012+10+($O1012*0.2)+(($O1012+10+($O1012*0.2))*$P1012))*0.05),0)</f>
+        <v/>
+      </c>
+      <c r="R1012" t="n">
+        <v>499</v>
+      </c>
+      <c r="S1012" t="n">
+        <v>499</v>
+      </c>
+      <c r="T1012" t="inlineStr">
+        <is>
+          <t>PDE26_C75AC4103313</t>
+        </is>
+      </c>
+    </row>
+    <row r="1013">
+      <c r="A1013" t="n">
+        <v>53</v>
+      </c>
+      <c r="B1013" t="inlineStr">
+        <is>
+          <t>Everyday</t>
+        </is>
+      </c>
+      <c r="C1013" t="inlineStr">
+        <is>
+          <t>TESTDEL_A1CF0A</t>
+        </is>
+      </c>
+      <c r="D1013" t="inlineStr">
+        <is>
+          <t>Women</t>
+        </is>
+      </c>
+      <c r="E1013" t="inlineStr">
+        <is>
+          <t>Nightdress</t>
+        </is>
+      </c>
+      <c r="F1013" t="inlineStr">
+        <is>
+          <t>Maxi</t>
+        </is>
+      </c>
+      <c r="G1013" t="inlineStr">
+        <is>
+          <t>SINGLE DRESS</t>
+        </is>
+      </c>
+      <c r="H1013" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="I1013" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="J1013" t="n">
+        <v>1</v>
+      </c>
+      <c r="K1013" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="L1013" t="inlineStr">
+        <is>
+          <t>XXL</t>
+        </is>
+      </c>
+      <c r="M1013" t="n">
+        <v>1</v>
+      </c>
+      <c r="N1013" t="inlineStr">
+        <is>
+          <t>TESTDEL_A1CF0A103813</t>
+        </is>
+      </c>
+      <c r="O1013" t="n">
+        <v>150</v>
+      </c>
+      <c r="P1013" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="Q1013">
+        <f>ROUND($O1013+10+($O1013*0.2)+(($O1013+10+($O1013*0.2))*$P1013)+(($O1013+10+($O1013*0.2)+(($O1013+10+($O1013*0.2))*$P1013))*0.05),0)</f>
+        <v/>
+      </c>
+      <c r="R1013" t="n">
+        <v>499</v>
+      </c>
+      <c r="S1013" t="n">
+        <v>499</v>
+      </c>
+      <c r="T1013" t="inlineStr">
+        <is>
+          <t>PTESTDEL_A1CF0A103813</t>
+        </is>
+      </c>
+    </row>
+    <row r="1014">
+      <c r="A1014" t="n">
+        <v>53</v>
+      </c>
+      <c r="B1014" t="inlineStr">
+        <is>
+          <t>Everyday</t>
+        </is>
+      </c>
+      <c r="C1014" t="inlineStr">
+        <is>
+          <t>TESTIMG_AE9AB0</t>
+        </is>
+      </c>
+      <c r="D1014" t="inlineStr">
+        <is>
+          <t>Nighty</t>
+        </is>
+      </c>
+      <c r="E1014" t="inlineStr">
+        <is>
+          <t>Sleeveless</t>
+        </is>
+      </c>
+      <c r="F1014" t="inlineStr">
+        <is>
+          <t>Square Neck</t>
+        </is>
+      </c>
+      <c r="G1014" t="inlineStr">
+        <is>
+          <t>SINGLE DRESS</t>
+        </is>
+      </c>
+      <c r="H1014" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="I1014" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="J1014" t="n">
+        <v>1</v>
+      </c>
+      <c r="K1014" t="inlineStr">
+        <is>
+          <t>Blue</t>
+        </is>
+      </c>
+      <c r="L1014" t="inlineStr">
+        <is>
+          <t>XXL</t>
+        </is>
+      </c>
+      <c r="M1014" t="n">
+        <v>1</v>
+      </c>
+      <c r="N1014" t="inlineStr">
+        <is>
+          <t>TESTIMG_AE9AB0103613</t>
+        </is>
+      </c>
+      <c r="O1014" t="n">
+        <v>185</v>
+      </c>
+      <c r="P1014" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="Q1014">
+        <f>ROUND($O1014+10+($O1014*0.2)+(($O1014+10+($O1014*0.2))*$P1014)+(($O1014+10+($O1014*0.2)+(($O1014+10+($O1014*0.2))*$P1014))*0.05),0)</f>
+        <v/>
+      </c>
+      <c r="R1014" t="n">
+        <v>499</v>
+      </c>
+      <c r="S1014" t="n">
+        <v>499</v>
+      </c>
+      <c r="T1014" t="inlineStr">
+        <is>
+          <t>PTESTIMG_AE9AB0103613</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(returns): implement editable Meesho SPF claim settlement and reconciliation tracking
</commit_message>
<xml_diff>
--- a/Barcode Master.xlsx
+++ b/Barcode Master.xlsx
@@ -995,7 +995,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z1014"/>
+  <dimension ref="A1:Z1052"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1" outlineLevelRow="1"/>
   <cols>
     <col width="9.33203125" customWidth="1" min="1" max="1"/>
@@ -32977,6 +32977,3312 @@
       <c r="T1014" t="inlineStr">
         <is>
           <t>PTESTIMG_AE9AB0103613</t>
+        </is>
+      </c>
+    </row>
+    <row r="1015">
+      <c r="A1015" t="n">
+        <v>54</v>
+      </c>
+      <c r="B1015" t="inlineStr">
+        <is>
+          <t>Everyday</t>
+        </is>
+      </c>
+      <c r="C1015" t="inlineStr">
+        <is>
+          <t>DE26_898300</t>
+        </is>
+      </c>
+      <c r="D1015" t="inlineStr">
+        <is>
+          <t>Nighty</t>
+        </is>
+      </c>
+      <c r="E1015" t="inlineStr">
+        <is>
+          <t>Sleeveless</t>
+        </is>
+      </c>
+      <c r="F1015" t="inlineStr">
+        <is>
+          <t>Square Neck</t>
+        </is>
+      </c>
+      <c r="G1015" t="inlineStr">
+        <is>
+          <t>SINGLE DRESS</t>
+        </is>
+      </c>
+      <c r="H1015" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="I1015" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="J1015" t="n">
+        <v>1</v>
+      </c>
+      <c r="K1015" t="inlineStr">
+        <is>
+          <t>Teal</t>
+        </is>
+      </c>
+      <c r="L1015" t="inlineStr">
+        <is>
+          <t>XXL</t>
+        </is>
+      </c>
+      <c r="M1015" t="n">
+        <v>1</v>
+      </c>
+      <c r="N1015" t="inlineStr">
+        <is>
+          <t>DE26_898300103313</t>
+        </is>
+      </c>
+      <c r="O1015" t="n">
+        <v>210</v>
+      </c>
+      <c r="P1015" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="Q1015">
+        <f>ROUND($O1015+10+($O1015*0.2)+(($O1015+10+($O1015*0.2))*$P1015)+(($O1015+10+($O1015*0.2)+(($O1015+10+($O1015*0.2))*$P1015))*0.05),0)</f>
+        <v/>
+      </c>
+      <c r="R1015" t="n">
+        <v>499</v>
+      </c>
+      <c r="S1015" t="n">
+        <v>499</v>
+      </c>
+      <c r="T1015" t="inlineStr">
+        <is>
+          <t>PDE26_898300103313</t>
+        </is>
+      </c>
+    </row>
+    <row r="1016">
+      <c r="A1016" t="n">
+        <v>55</v>
+      </c>
+      <c r="B1016" t="inlineStr">
+        <is>
+          <t>Everyday</t>
+        </is>
+      </c>
+      <c r="C1016" t="inlineStr">
+        <is>
+          <t>TESTDEL_CAD1F1</t>
+        </is>
+      </c>
+      <c r="D1016" t="inlineStr">
+        <is>
+          <t>Women</t>
+        </is>
+      </c>
+      <c r="E1016" t="inlineStr">
+        <is>
+          <t>Nightdress</t>
+        </is>
+      </c>
+      <c r="F1016" t="inlineStr">
+        <is>
+          <t>Maxi</t>
+        </is>
+      </c>
+      <c r="G1016" t="inlineStr">
+        <is>
+          <t>SINGLE DRESS</t>
+        </is>
+      </c>
+      <c r="H1016" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="I1016" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="J1016" t="n">
+        <v>1</v>
+      </c>
+      <c r="K1016" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="L1016" t="inlineStr">
+        <is>
+          <t>XXL</t>
+        </is>
+      </c>
+      <c r="M1016" t="n">
+        <v>1</v>
+      </c>
+      <c r="N1016" t="inlineStr">
+        <is>
+          <t>TESTDEL_CAD1F1103813</t>
+        </is>
+      </c>
+      <c r="O1016" t="n">
+        <v>150</v>
+      </c>
+      <c r="P1016" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="Q1016">
+        <f>ROUND($O1016+10+($O1016*0.2)+(($O1016+10+($O1016*0.2))*$P1016)+(($O1016+10+($O1016*0.2)+(($O1016+10+($O1016*0.2))*$P1016))*0.05),0)</f>
+        <v/>
+      </c>
+      <c r="R1016" t="n">
+        <v>499</v>
+      </c>
+      <c r="S1016" t="n">
+        <v>499</v>
+      </c>
+      <c r="T1016" t="inlineStr">
+        <is>
+          <t>PTESTDEL_CAD1F1103813</t>
+        </is>
+      </c>
+    </row>
+    <row r="1017">
+      <c r="A1017" t="n">
+        <v>55</v>
+      </c>
+      <c r="B1017" t="inlineStr">
+        <is>
+          <t>Everyday</t>
+        </is>
+      </c>
+      <c r="C1017" t="inlineStr">
+        <is>
+          <t>TESTIMG_5434EA</t>
+        </is>
+      </c>
+      <c r="D1017" t="inlineStr">
+        <is>
+          <t>Nighty</t>
+        </is>
+      </c>
+      <c r="E1017" t="inlineStr">
+        <is>
+          <t>Sleeveless</t>
+        </is>
+      </c>
+      <c r="F1017" t="inlineStr">
+        <is>
+          <t>Square Neck</t>
+        </is>
+      </c>
+      <c r="G1017" t="inlineStr">
+        <is>
+          <t>SINGLE DRESS</t>
+        </is>
+      </c>
+      <c r="H1017" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="I1017" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="J1017" t="n">
+        <v>1</v>
+      </c>
+      <c r="K1017" t="inlineStr">
+        <is>
+          <t>Blue</t>
+        </is>
+      </c>
+      <c r="L1017" t="inlineStr">
+        <is>
+          <t>XXL</t>
+        </is>
+      </c>
+      <c r="M1017" t="n">
+        <v>1</v>
+      </c>
+      <c r="N1017" t="inlineStr">
+        <is>
+          <t>TESTIMG_5434EA103613</t>
+        </is>
+      </c>
+      <c r="O1017" t="n">
+        <v>185</v>
+      </c>
+      <c r="P1017" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="Q1017">
+        <f>ROUND($O1017+10+($O1017*0.2)+(($O1017+10+($O1017*0.2))*$P1017)+(($O1017+10+($O1017*0.2)+(($O1017+10+($O1017*0.2))*$P1017))*0.05),0)</f>
+        <v/>
+      </c>
+      <c r="R1017" t="n">
+        <v>499</v>
+      </c>
+      <c r="S1017" t="n">
+        <v>499</v>
+      </c>
+      <c r="T1017" t="inlineStr">
+        <is>
+          <t>PTESTIMG_5434EA103613</t>
+        </is>
+      </c>
+    </row>
+    <row r="1018">
+      <c r="A1018" t="n">
+        <v>43</v>
+      </c>
+      <c r="B1018" t="inlineStr">
+        <is>
+          <t>Everyday</t>
+        </is>
+      </c>
+      <c r="C1018" t="inlineStr">
+        <is>
+          <t>DE26011B</t>
+        </is>
+      </c>
+      <c r="D1018" t="inlineStr">
+        <is>
+          <t>Nighty</t>
+        </is>
+      </c>
+      <c r="E1018" t="inlineStr">
+        <is>
+          <t>Short Sleeves</t>
+        </is>
+      </c>
+      <c r="F1018" t="inlineStr">
+        <is>
+          <t>Square Neck</t>
+        </is>
+      </c>
+      <c r="G1018" t="inlineStr">
+        <is>
+          <t>SINGLE DRESS</t>
+        </is>
+      </c>
+      <c r="H1018" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="I1018" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="J1018" t="n">
+        <v>1</v>
+      </c>
+      <c r="K1018" t="inlineStr">
+        <is>
+          <t>Brown</t>
+        </is>
+      </c>
+      <c r="L1018" t="inlineStr">
+        <is>
+          <t>XXL</t>
+        </is>
+      </c>
+      <c r="M1018" t="n">
+        <v>1</v>
+      </c>
+      <c r="N1018" t="inlineStr">
+        <is>
+          <t>DE26011B104013</t>
+        </is>
+      </c>
+      <c r="O1018" t="n">
+        <v>185</v>
+      </c>
+      <c r="P1018" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="Q1018">
+        <f>ROUND($O1018+10+($O1018*0.2)+(($O1018+10+($O1018*0.2))*$P1018)+(($O1018+10+($O1018*0.2)+(($O1018+10+($O1018*0.2))*$P1018))*0.05),0)</f>
+        <v/>
+      </c>
+      <c r="R1018" t="n">
+        <v>449</v>
+      </c>
+      <c r="S1018" t="n">
+        <v>449</v>
+      </c>
+      <c r="T1018" t="inlineStr">
+        <is>
+          <t>PDE26011B104013</t>
+        </is>
+      </c>
+    </row>
+    <row r="1019">
+      <c r="A1019" t="n">
+        <v>56</v>
+      </c>
+      <c r="B1019" t="inlineStr">
+        <is>
+          <t>Everyday</t>
+        </is>
+      </c>
+      <c r="C1019" t="inlineStr">
+        <is>
+          <t>DE26_94DF66</t>
+        </is>
+      </c>
+      <c r="D1019" t="inlineStr">
+        <is>
+          <t>Nighty</t>
+        </is>
+      </c>
+      <c r="E1019" t="inlineStr">
+        <is>
+          <t>Sleeveless</t>
+        </is>
+      </c>
+      <c r="F1019" t="inlineStr">
+        <is>
+          <t>Square Neck</t>
+        </is>
+      </c>
+      <c r="G1019" t="inlineStr">
+        <is>
+          <t>SINGLE DRESS</t>
+        </is>
+      </c>
+      <c r="H1019" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="I1019" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="J1019" t="n">
+        <v>1</v>
+      </c>
+      <c r="K1019" t="inlineStr">
+        <is>
+          <t>Teal</t>
+        </is>
+      </c>
+      <c r="L1019" t="inlineStr">
+        <is>
+          <t>XXL</t>
+        </is>
+      </c>
+      <c r="M1019" t="n">
+        <v>1</v>
+      </c>
+      <c r="N1019" t="inlineStr">
+        <is>
+          <t>DE26_94DF66103313</t>
+        </is>
+      </c>
+      <c r="O1019" t="n">
+        <v>210</v>
+      </c>
+      <c r="P1019" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="Q1019">
+        <f>ROUND($O1019+10+($O1019*0.2)+(($O1019+10+($O1019*0.2))*$P1019)+(($O1019+10+($O1019*0.2)+(($O1019+10+($O1019*0.2))*$P1019))*0.05),0)</f>
+        <v/>
+      </c>
+      <c r="R1019" t="n">
+        <v>499</v>
+      </c>
+      <c r="S1019" t="n">
+        <v>499</v>
+      </c>
+      <c r="T1019" t="inlineStr">
+        <is>
+          <t>PDE26_94DF66103313</t>
+        </is>
+      </c>
+    </row>
+    <row r="1020">
+      <c r="A1020" t="n">
+        <v>57</v>
+      </c>
+      <c r="B1020" t="inlineStr">
+        <is>
+          <t>Everyday</t>
+        </is>
+      </c>
+      <c r="C1020" t="inlineStr">
+        <is>
+          <t>TESTDEL_2D6486</t>
+        </is>
+      </c>
+      <c r="D1020" t="inlineStr">
+        <is>
+          <t>Women</t>
+        </is>
+      </c>
+      <c r="E1020" t="inlineStr">
+        <is>
+          <t>Nightdress</t>
+        </is>
+      </c>
+      <c r="F1020" t="inlineStr">
+        <is>
+          <t>Maxi</t>
+        </is>
+      </c>
+      <c r="G1020" t="inlineStr">
+        <is>
+          <t>SINGLE DRESS</t>
+        </is>
+      </c>
+      <c r="H1020" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="I1020" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="J1020" t="n">
+        <v>1</v>
+      </c>
+      <c r="K1020" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="L1020" t="inlineStr">
+        <is>
+          <t>XXL</t>
+        </is>
+      </c>
+      <c r="M1020" t="n">
+        <v>1</v>
+      </c>
+      <c r="N1020" t="inlineStr">
+        <is>
+          <t>TESTDEL_2D6486103813</t>
+        </is>
+      </c>
+      <c r="O1020" t="n">
+        <v>150</v>
+      </c>
+      <c r="P1020" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="Q1020">
+        <f>ROUND($O1020+10+($O1020*0.2)+(($O1020+10+($O1020*0.2))*$P1020)+(($O1020+10+($O1020*0.2)+(($O1020+10+($O1020*0.2))*$P1020))*0.05),0)</f>
+        <v/>
+      </c>
+      <c r="R1020" t="n">
+        <v>499</v>
+      </c>
+      <c r="S1020" t="n">
+        <v>499</v>
+      </c>
+      <c r="T1020" t="inlineStr">
+        <is>
+          <t>PTESTDEL_2D6486103813</t>
+        </is>
+      </c>
+    </row>
+    <row r="1021">
+      <c r="A1021" t="n">
+        <v>57</v>
+      </c>
+      <c r="B1021" t="inlineStr">
+        <is>
+          <t>Everyday</t>
+        </is>
+      </c>
+      <c r="C1021" t="inlineStr">
+        <is>
+          <t>TESTIMG_25027C</t>
+        </is>
+      </c>
+      <c r="D1021" t="inlineStr">
+        <is>
+          <t>Nighty</t>
+        </is>
+      </c>
+      <c r="E1021" t="inlineStr">
+        <is>
+          <t>Sleeveless</t>
+        </is>
+      </c>
+      <c r="F1021" t="inlineStr">
+        <is>
+          <t>Square Neck</t>
+        </is>
+      </c>
+      <c r="G1021" t="inlineStr">
+        <is>
+          <t>SINGLE DRESS</t>
+        </is>
+      </c>
+      <c r="H1021" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="I1021" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="J1021" t="n">
+        <v>1</v>
+      </c>
+      <c r="K1021" t="inlineStr">
+        <is>
+          <t>Blue</t>
+        </is>
+      </c>
+      <c r="L1021" t="inlineStr">
+        <is>
+          <t>XXL</t>
+        </is>
+      </c>
+      <c r="M1021" t="n">
+        <v>1</v>
+      </c>
+      <c r="N1021" t="inlineStr">
+        <is>
+          <t>TESTIMG_25027C103613</t>
+        </is>
+      </c>
+      <c r="O1021" t="n">
+        <v>185</v>
+      </c>
+      <c r="P1021" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="Q1021">
+        <f>ROUND($O1021+10+($O1021*0.2)+(($O1021+10+($O1021*0.2))*$P1021)+(($O1021+10+($O1021*0.2)+(($O1021+10+($O1021*0.2))*$P1021))*0.05),0)</f>
+        <v/>
+      </c>
+      <c r="R1021" t="n">
+        <v>499</v>
+      </c>
+      <c r="S1021" t="n">
+        <v>499</v>
+      </c>
+      <c r="T1021" t="inlineStr">
+        <is>
+          <t>PTESTIMG_25027C103613</t>
+        </is>
+      </c>
+    </row>
+    <row r="1022">
+      <c r="A1022" t="n">
+        <v>44</v>
+      </c>
+      <c r="B1022" t="inlineStr">
+        <is>
+          <t>Everyday</t>
+        </is>
+      </c>
+      <c r="C1022" t="inlineStr">
+        <is>
+          <t>DE26011G</t>
+        </is>
+      </c>
+      <c r="D1022" t="inlineStr">
+        <is>
+          <t>Nighty</t>
+        </is>
+      </c>
+      <c r="E1022" t="inlineStr">
+        <is>
+          <t>Short Sleeves</t>
+        </is>
+      </c>
+      <c r="F1022" t="inlineStr">
+        <is>
+          <t>Square Neck</t>
+        </is>
+      </c>
+      <c r="G1022" t="inlineStr">
+        <is>
+          <t>SINGLE DRESS</t>
+        </is>
+      </c>
+      <c r="H1022" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="I1022" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="J1022" t="n">
+        <v>1</v>
+      </c>
+      <c r="K1022" t="inlineStr">
+        <is>
+          <t>Green</t>
+        </is>
+      </c>
+      <c r="L1022" t="inlineStr">
+        <is>
+          <t>XXL</t>
+        </is>
+      </c>
+      <c r="M1022" t="n">
+        <v>1</v>
+      </c>
+      <c r="N1022" t="inlineStr">
+        <is>
+          <t>DE26011G103413</t>
+        </is>
+      </c>
+      <c r="O1022" t="n">
+        <v>185</v>
+      </c>
+      <c r="P1022" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="Q1022">
+        <f>ROUND($O1022+10+($O1022*0.2)+(($O1022+10+($O1022*0.2))*$P1022)+(($O1022+10+($O1022*0.2)+(($O1022+10+($O1022*0.2))*$P1022))*0.05),0)</f>
+        <v/>
+      </c>
+      <c r="R1022" t="n">
+        <v>449</v>
+      </c>
+      <c r="S1022" t="n">
+        <v>449</v>
+      </c>
+      <c r="T1022" t="inlineStr">
+        <is>
+          <t>PDE26011G103413</t>
+        </is>
+      </c>
+    </row>
+    <row r="1023">
+      <c r="A1023" t="n">
+        <v>45</v>
+      </c>
+      <c r="B1023" t="inlineStr">
+        <is>
+          <t>Everyday</t>
+        </is>
+      </c>
+      <c r="C1023" t="inlineStr">
+        <is>
+          <t>DE26011P</t>
+        </is>
+      </c>
+      <c r="D1023" t="inlineStr">
+        <is>
+          <t>Nighty</t>
+        </is>
+      </c>
+      <c r="E1023" t="inlineStr">
+        <is>
+          <t>Short Sleeves</t>
+        </is>
+      </c>
+      <c r="F1023" t="inlineStr">
+        <is>
+          <t>Square Neck</t>
+        </is>
+      </c>
+      <c r="G1023" t="inlineStr">
+        <is>
+          <t>SINGLE DRESS</t>
+        </is>
+      </c>
+      <c r="H1023" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="I1023" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="J1023" t="n">
+        <v>1</v>
+      </c>
+      <c r="K1023" t="inlineStr">
+        <is>
+          <t>Pink</t>
+        </is>
+      </c>
+      <c r="L1023" t="inlineStr">
+        <is>
+          <t>XXL</t>
+        </is>
+      </c>
+      <c r="M1023" t="n">
+        <v>1</v>
+      </c>
+      <c r="N1023" t="inlineStr">
+        <is>
+          <t>DE26011P101413</t>
+        </is>
+      </c>
+      <c r="O1023" t="n">
+        <v>185</v>
+      </c>
+      <c r="P1023" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="Q1023">
+        <f>ROUND($O1023+10+($O1023*0.2)+(($O1023+10+($O1023*0.2))*$P1023)+(($O1023+10+($O1023*0.2)+(($O1023+10+($O1023*0.2))*$P1023))*0.05),0)</f>
+        <v/>
+      </c>
+      <c r="R1023" t="n">
+        <v>449</v>
+      </c>
+      <c r="S1023" t="n">
+        <v>449</v>
+      </c>
+      <c r="T1023" t="inlineStr">
+        <is>
+          <t>PDE26011P101413</t>
+        </is>
+      </c>
+    </row>
+    <row r="1024">
+      <c r="A1024" t="n">
+        <v>46</v>
+      </c>
+      <c r="B1024" t="inlineStr">
+        <is>
+          <t>Everyday</t>
+        </is>
+      </c>
+      <c r="C1024" t="inlineStr">
+        <is>
+          <t>DE26011R</t>
+        </is>
+      </c>
+      <c r="D1024" t="inlineStr">
+        <is>
+          <t>Nighty</t>
+        </is>
+      </c>
+      <c r="E1024" t="inlineStr">
+        <is>
+          <t>Short Sleeves</t>
+        </is>
+      </c>
+      <c r="F1024" t="inlineStr">
+        <is>
+          <t>Square Neck</t>
+        </is>
+      </c>
+      <c r="G1024" t="inlineStr">
+        <is>
+          <t>SINGLE DRESS</t>
+        </is>
+      </c>
+      <c r="H1024" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="I1024" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="J1024" t="n">
+        <v>1</v>
+      </c>
+      <c r="K1024" t="inlineStr">
+        <is>
+          <t>Red</t>
+        </is>
+      </c>
+      <c r="L1024" t="inlineStr">
+        <is>
+          <t>XXL</t>
+        </is>
+      </c>
+      <c r="M1024" t="n">
+        <v>1</v>
+      </c>
+      <c r="N1024" t="inlineStr">
+        <is>
+          <t>DE26011R101213</t>
+        </is>
+      </c>
+      <c r="O1024" t="n">
+        <v>185</v>
+      </c>
+      <c r="P1024" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="Q1024">
+        <f>ROUND($O1024+10+($O1024*0.2)+(($O1024+10+($O1024*0.2))*$P1024)+(($O1024+10+($O1024*0.2)+(($O1024+10+($O1024*0.2))*$P1024))*0.05),0)</f>
+        <v/>
+      </c>
+      <c r="R1024" t="n">
+        <v>449</v>
+      </c>
+      <c r="S1024" t="n">
+        <v>449</v>
+      </c>
+      <c r="T1024" t="inlineStr">
+        <is>
+          <t>PDE26011R101213</t>
+        </is>
+      </c>
+    </row>
+    <row r="1025">
+      <c r="A1025" t="n">
+        <v>58</v>
+      </c>
+      <c r="B1025" t="inlineStr">
+        <is>
+          <t>Everyday</t>
+        </is>
+      </c>
+      <c r="C1025" t="inlineStr">
+        <is>
+          <t>DE26_034F2B</t>
+        </is>
+      </c>
+      <c r="D1025" t="inlineStr">
+        <is>
+          <t>Nighty</t>
+        </is>
+      </c>
+      <c r="E1025" t="inlineStr">
+        <is>
+          <t>Sleeveless</t>
+        </is>
+      </c>
+      <c r="F1025" t="inlineStr">
+        <is>
+          <t>Square Neck</t>
+        </is>
+      </c>
+      <c r="G1025" t="inlineStr">
+        <is>
+          <t>SINGLE DRESS</t>
+        </is>
+      </c>
+      <c r="H1025" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="I1025" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="J1025" t="n">
+        <v>1</v>
+      </c>
+      <c r="K1025" t="inlineStr">
+        <is>
+          <t>Teal</t>
+        </is>
+      </c>
+      <c r="L1025" t="inlineStr">
+        <is>
+          <t>XXL</t>
+        </is>
+      </c>
+      <c r="M1025" t="n">
+        <v>1</v>
+      </c>
+      <c r="N1025" t="inlineStr">
+        <is>
+          <t>DE26_034F2B103313</t>
+        </is>
+      </c>
+      <c r="O1025" t="n">
+        <v>210</v>
+      </c>
+      <c r="P1025" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="Q1025">
+        <f>ROUND($O1025+10+($O1025*0.2)+(($O1025+10+($O1025*0.2))*$P1025)+(($O1025+10+($O1025*0.2)+(($O1025+10+($O1025*0.2))*$P1025))*0.05),0)</f>
+        <v/>
+      </c>
+      <c r="R1025" t="n">
+        <v>499</v>
+      </c>
+      <c r="S1025" t="n">
+        <v>499</v>
+      </c>
+      <c r="T1025" t="inlineStr">
+        <is>
+          <t>PDE26_034F2B103313</t>
+        </is>
+      </c>
+    </row>
+    <row r="1026">
+      <c r="A1026" t="n">
+        <v>59</v>
+      </c>
+      <c r="B1026" t="inlineStr">
+        <is>
+          <t>Everyday</t>
+        </is>
+      </c>
+      <c r="C1026" t="inlineStr">
+        <is>
+          <t>TESTDEL_9F1C59</t>
+        </is>
+      </c>
+      <c r="D1026" t="inlineStr">
+        <is>
+          <t>Women</t>
+        </is>
+      </c>
+      <c r="E1026" t="inlineStr">
+        <is>
+          <t>Nightdress</t>
+        </is>
+      </c>
+      <c r="F1026" t="inlineStr">
+        <is>
+          <t>Maxi</t>
+        </is>
+      </c>
+      <c r="G1026" t="inlineStr">
+        <is>
+          <t>SINGLE DRESS</t>
+        </is>
+      </c>
+      <c r="H1026" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="I1026" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="J1026" t="n">
+        <v>1</v>
+      </c>
+      <c r="K1026" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="L1026" t="inlineStr">
+        <is>
+          <t>XXL</t>
+        </is>
+      </c>
+      <c r="M1026" t="n">
+        <v>1</v>
+      </c>
+      <c r="N1026" t="inlineStr">
+        <is>
+          <t>TESTDEL_9F1C59103813</t>
+        </is>
+      </c>
+      <c r="O1026" t="n">
+        <v>150</v>
+      </c>
+      <c r="P1026" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="Q1026">
+        <f>ROUND($O1026+10+($O1026*0.2)+(($O1026+10+($O1026*0.2))*$P1026)+(($O1026+10+($O1026*0.2)+(($O1026+10+($O1026*0.2))*$P1026))*0.05),0)</f>
+        <v/>
+      </c>
+      <c r="R1026" t="n">
+        <v>499</v>
+      </c>
+      <c r="S1026" t="n">
+        <v>499</v>
+      </c>
+      <c r="T1026" t="inlineStr">
+        <is>
+          <t>PTESTDEL_9F1C59103813</t>
+        </is>
+      </c>
+    </row>
+    <row r="1027">
+      <c r="A1027" t="n">
+        <v>59</v>
+      </c>
+      <c r="B1027" t="inlineStr">
+        <is>
+          <t>Everyday</t>
+        </is>
+      </c>
+      <c r="C1027" t="inlineStr">
+        <is>
+          <t>TESTIMG_89EBE7</t>
+        </is>
+      </c>
+      <c r="D1027" t="inlineStr">
+        <is>
+          <t>Nighty</t>
+        </is>
+      </c>
+      <c r="E1027" t="inlineStr">
+        <is>
+          <t>Sleeveless</t>
+        </is>
+      </c>
+      <c r="F1027" t="inlineStr">
+        <is>
+          <t>Square Neck</t>
+        </is>
+      </c>
+      <c r="G1027" t="inlineStr">
+        <is>
+          <t>SINGLE DRESS</t>
+        </is>
+      </c>
+      <c r="H1027" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="I1027" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="J1027" t="n">
+        <v>1</v>
+      </c>
+      <c r="K1027" t="inlineStr">
+        <is>
+          <t>Blue</t>
+        </is>
+      </c>
+      <c r="L1027" t="inlineStr">
+        <is>
+          <t>XXL</t>
+        </is>
+      </c>
+      <c r="M1027" t="n">
+        <v>1</v>
+      </c>
+      <c r="N1027" t="inlineStr">
+        <is>
+          <t>TESTIMG_89EBE7103613</t>
+        </is>
+      </c>
+      <c r="O1027" t="n">
+        <v>185</v>
+      </c>
+      <c r="P1027" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="Q1027">
+        <f>ROUND($O1027+10+($O1027*0.2)+(($O1027+10+($O1027*0.2))*$P1027)+(($O1027+10+($O1027*0.2)+(($O1027+10+($O1027*0.2))*$P1027))*0.05),0)</f>
+        <v/>
+      </c>
+      <c r="R1027" t="n">
+        <v>499</v>
+      </c>
+      <c r="S1027" t="n">
+        <v>499</v>
+      </c>
+      <c r="T1027" t="inlineStr">
+        <is>
+          <t>PTESTIMG_89EBE7103613</t>
+        </is>
+      </c>
+    </row>
+    <row r="1028">
+      <c r="A1028" t="n">
+        <v>60</v>
+      </c>
+      <c r="B1028" t="inlineStr">
+        <is>
+          <t>Everyday</t>
+        </is>
+      </c>
+      <c r="C1028" t="inlineStr">
+        <is>
+          <t>DE26_A881F3</t>
+        </is>
+      </c>
+      <c r="D1028" t="inlineStr">
+        <is>
+          <t>Nighty</t>
+        </is>
+      </c>
+      <c r="E1028" t="inlineStr">
+        <is>
+          <t>Sleeveless</t>
+        </is>
+      </c>
+      <c r="F1028" t="inlineStr">
+        <is>
+          <t>Square Neck</t>
+        </is>
+      </c>
+      <c r="G1028" t="inlineStr">
+        <is>
+          <t>SINGLE DRESS</t>
+        </is>
+      </c>
+      <c r="H1028" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="I1028" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="J1028" t="n">
+        <v>1</v>
+      </c>
+      <c r="K1028" t="inlineStr">
+        <is>
+          <t>Teal</t>
+        </is>
+      </c>
+      <c r="L1028" t="inlineStr">
+        <is>
+          <t>XXL</t>
+        </is>
+      </c>
+      <c r="M1028" t="n">
+        <v>1</v>
+      </c>
+      <c r="N1028" t="inlineStr">
+        <is>
+          <t>DE26_A881F3103313</t>
+        </is>
+      </c>
+      <c r="O1028" t="n">
+        <v>210</v>
+      </c>
+      <c r="P1028" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="Q1028">
+        <f>ROUND($O1028+10+($O1028*0.2)+(($O1028+10+($O1028*0.2))*$P1028)+(($O1028+10+($O1028*0.2)+(($O1028+10+($O1028*0.2))*$P1028))*0.05),0)</f>
+        <v/>
+      </c>
+      <c r="R1028" t="n">
+        <v>499</v>
+      </c>
+      <c r="S1028" t="n">
+        <v>499</v>
+      </c>
+      <c r="T1028" t="inlineStr">
+        <is>
+          <t>PDE26_A881F3103313</t>
+        </is>
+      </c>
+    </row>
+    <row r="1029">
+      <c r="A1029" t="n">
+        <v>61</v>
+      </c>
+      <c r="B1029" t="inlineStr">
+        <is>
+          <t>Everyday</t>
+        </is>
+      </c>
+      <c r="C1029" t="inlineStr">
+        <is>
+          <t>TESTDEL_E96E1F</t>
+        </is>
+      </c>
+      <c r="D1029" t="inlineStr">
+        <is>
+          <t>Women</t>
+        </is>
+      </c>
+      <c r="E1029" t="inlineStr">
+        <is>
+          <t>Nightdress</t>
+        </is>
+      </c>
+      <c r="F1029" t="inlineStr">
+        <is>
+          <t>Maxi</t>
+        </is>
+      </c>
+      <c r="G1029" t="inlineStr">
+        <is>
+          <t>SINGLE DRESS</t>
+        </is>
+      </c>
+      <c r="H1029" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="I1029" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="J1029" t="n">
+        <v>1</v>
+      </c>
+      <c r="K1029" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="L1029" t="inlineStr">
+        <is>
+          <t>XXL</t>
+        </is>
+      </c>
+      <c r="M1029" t="n">
+        <v>1</v>
+      </c>
+      <c r="N1029" t="inlineStr">
+        <is>
+          <t>TESTDEL_E96E1F103813</t>
+        </is>
+      </c>
+      <c r="O1029" t="n">
+        <v>150</v>
+      </c>
+      <c r="P1029" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="Q1029">
+        <f>ROUND($O1029+10+($O1029*0.2)+(($O1029+10+($O1029*0.2))*$P1029)+(($O1029+10+($O1029*0.2)+(($O1029+10+($O1029*0.2))*$P1029))*0.05),0)</f>
+        <v/>
+      </c>
+      <c r="R1029" t="n">
+        <v>499</v>
+      </c>
+      <c r="S1029" t="n">
+        <v>499</v>
+      </c>
+      <c r="T1029" t="inlineStr">
+        <is>
+          <t>PTESTDEL_E96E1F103813</t>
+        </is>
+      </c>
+    </row>
+    <row r="1030">
+      <c r="A1030" t="n">
+        <v>61</v>
+      </c>
+      <c r="B1030" t="inlineStr">
+        <is>
+          <t>Everyday</t>
+        </is>
+      </c>
+      <c r="C1030" t="inlineStr">
+        <is>
+          <t>TESTIMG_83797E</t>
+        </is>
+      </c>
+      <c r="D1030" t="inlineStr">
+        <is>
+          <t>Nighty</t>
+        </is>
+      </c>
+      <c r="E1030" t="inlineStr">
+        <is>
+          <t>Sleeveless</t>
+        </is>
+      </c>
+      <c r="F1030" t="inlineStr">
+        <is>
+          <t>Square Neck</t>
+        </is>
+      </c>
+      <c r="G1030" t="inlineStr">
+        <is>
+          <t>SINGLE DRESS</t>
+        </is>
+      </c>
+      <c r="H1030" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="I1030" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="J1030" t="n">
+        <v>1</v>
+      </c>
+      <c r="K1030" t="inlineStr">
+        <is>
+          <t>Blue</t>
+        </is>
+      </c>
+      <c r="L1030" t="inlineStr">
+        <is>
+          <t>XXL</t>
+        </is>
+      </c>
+      <c r="M1030" t="n">
+        <v>1</v>
+      </c>
+      <c r="N1030" t="inlineStr">
+        <is>
+          <t>TESTIMG_83797E103613</t>
+        </is>
+      </c>
+      <c r="O1030" t="n">
+        <v>185</v>
+      </c>
+      <c r="P1030" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="Q1030">
+        <f>ROUND($O1030+10+($O1030*0.2)+(($O1030+10+($O1030*0.2))*$P1030)+(($O1030+10+($O1030*0.2)+(($O1030+10+($O1030*0.2))*$P1030))*0.05),0)</f>
+        <v/>
+      </c>
+      <c r="R1030" t="n">
+        <v>499</v>
+      </c>
+      <c r="S1030" t="n">
+        <v>499</v>
+      </c>
+      <c r="T1030" t="inlineStr">
+        <is>
+          <t>PTESTIMG_83797E103613</t>
+        </is>
+      </c>
+    </row>
+    <row r="1031">
+      <c r="A1031" t="n">
+        <v>47</v>
+      </c>
+      <c r="B1031" t="inlineStr">
+        <is>
+          <t>Everyday</t>
+        </is>
+      </c>
+      <c r="C1031" t="inlineStr">
+        <is>
+          <t>DE26010B</t>
+        </is>
+      </c>
+      <c r="D1031" t="inlineStr">
+        <is>
+          <t>Nighty</t>
+        </is>
+      </c>
+      <c r="E1031" t="inlineStr">
+        <is>
+          <t>Short Sleeves</t>
+        </is>
+      </c>
+      <c r="F1031" t="inlineStr">
+        <is>
+          <t>Square Neck</t>
+        </is>
+      </c>
+      <c r="G1031" t="inlineStr">
+        <is>
+          <t>SINGLE DRESS</t>
+        </is>
+      </c>
+      <c r="H1031" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="I1031" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="J1031" t="n">
+        <v>1</v>
+      </c>
+      <c r="K1031" t="inlineStr">
+        <is>
+          <t>Brown</t>
+        </is>
+      </c>
+      <c r="L1031" t="inlineStr">
+        <is>
+          <t>XXL</t>
+        </is>
+      </c>
+      <c r="M1031" t="n">
+        <v>1</v>
+      </c>
+      <c r="N1031" t="inlineStr">
+        <is>
+          <t>DE26010B104013</t>
+        </is>
+      </c>
+      <c r="O1031" t="n">
+        <v>185</v>
+      </c>
+      <c r="P1031" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="Q1031">
+        <f>ROUND($O1031+10+($O1031*0.2)+(($O1031+10+($O1031*0.2))*$P1031)+(($O1031+10+($O1031*0.2)+(($O1031+10+($O1031*0.2))*$P1031))*0.05),0)</f>
+        <v/>
+      </c>
+      <c r="R1031" t="n">
+        <v>449</v>
+      </c>
+      <c r="S1031" t="n">
+        <v>449</v>
+      </c>
+      <c r="T1031" t="inlineStr">
+        <is>
+          <t>PDE26010B104013</t>
+        </is>
+      </c>
+    </row>
+    <row r="1032">
+      <c r="A1032" t="n">
+        <v>48</v>
+      </c>
+      <c r="B1032" t="inlineStr">
+        <is>
+          <t>Everyday</t>
+        </is>
+      </c>
+      <c r="C1032" t="inlineStr">
+        <is>
+          <t>DE26010G</t>
+        </is>
+      </c>
+      <c r="D1032" t="inlineStr">
+        <is>
+          <t>Nighty</t>
+        </is>
+      </c>
+      <c r="E1032" t="inlineStr">
+        <is>
+          <t>Short Sleeves</t>
+        </is>
+      </c>
+      <c r="F1032" t="inlineStr">
+        <is>
+          <t>Square Neck</t>
+        </is>
+      </c>
+      <c r="G1032" t="inlineStr">
+        <is>
+          <t>SINGLE DRESS</t>
+        </is>
+      </c>
+      <c r="H1032" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="I1032" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="J1032" t="n">
+        <v>1</v>
+      </c>
+      <c r="K1032" t="inlineStr">
+        <is>
+          <t>Green</t>
+        </is>
+      </c>
+      <c r="L1032" t="inlineStr">
+        <is>
+          <t>XXL</t>
+        </is>
+      </c>
+      <c r="M1032" t="n">
+        <v>1</v>
+      </c>
+      <c r="N1032" t="inlineStr">
+        <is>
+          <t>DE26010G103413</t>
+        </is>
+      </c>
+      <c r="O1032" t="n">
+        <v>185</v>
+      </c>
+      <c r="P1032" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="Q1032">
+        <f>ROUND($O1032+10+($O1032*0.2)+(($O1032+10+($O1032*0.2))*$P1032)+(($O1032+10+($O1032*0.2)+(($O1032+10+($O1032*0.2))*$P1032))*0.05),0)</f>
+        <v/>
+      </c>
+      <c r="R1032" t="n">
+        <v>449</v>
+      </c>
+      <c r="S1032" t="n">
+        <v>449</v>
+      </c>
+      <c r="T1032" t="inlineStr">
+        <is>
+          <t>PDE26010G103413</t>
+        </is>
+      </c>
+    </row>
+    <row r="1033">
+      <c r="A1033" t="n">
+        <v>49</v>
+      </c>
+      <c r="B1033" t="inlineStr">
+        <is>
+          <t>Everyday</t>
+        </is>
+      </c>
+      <c r="C1033" t="inlineStr">
+        <is>
+          <t>DE26010M</t>
+        </is>
+      </c>
+      <c r="D1033" t="inlineStr">
+        <is>
+          <t>Nighty</t>
+        </is>
+      </c>
+      <c r="E1033" t="inlineStr">
+        <is>
+          <t>Short Sleeves</t>
+        </is>
+      </c>
+      <c r="F1033" t="inlineStr">
+        <is>
+          <t>Square Neck</t>
+        </is>
+      </c>
+      <c r="G1033" t="inlineStr">
+        <is>
+          <t>SINGLE DRESS</t>
+        </is>
+      </c>
+      <c r="H1033" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="I1033" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="J1033" t="n">
+        <v>1</v>
+      </c>
+      <c r="K1033" t="inlineStr">
+        <is>
+          <t>Maroon</t>
+        </is>
+      </c>
+      <c r="L1033" t="inlineStr">
+        <is>
+          <t>XXL</t>
+        </is>
+      </c>
+      <c r="M1033" t="n">
+        <v>1</v>
+      </c>
+      <c r="N1033" t="inlineStr">
+        <is>
+          <t>DE26010M103213</t>
+        </is>
+      </c>
+      <c r="O1033" t="n">
+        <v>185</v>
+      </c>
+      <c r="P1033" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="Q1033">
+        <f>ROUND($O1033+10+($O1033*0.2)+(($O1033+10+($O1033*0.2))*$P1033)+(($O1033+10+($O1033*0.2)+(($O1033+10+($O1033*0.2))*$P1033))*0.05),0)</f>
+        <v/>
+      </c>
+      <c r="R1033" t="n">
+        <v>449</v>
+      </c>
+      <c r="S1033" t="n">
+        <v>449</v>
+      </c>
+      <c r="T1033" t="inlineStr">
+        <is>
+          <t>PDE26010M103213</t>
+        </is>
+      </c>
+    </row>
+    <row r="1034">
+      <c r="A1034" t="n">
+        <v>50</v>
+      </c>
+      <c r="B1034" t="inlineStr">
+        <is>
+          <t>Everyday</t>
+        </is>
+      </c>
+      <c r="C1034" t="inlineStr">
+        <is>
+          <t>DE26010N</t>
+        </is>
+      </c>
+      <c r="D1034" t="inlineStr">
+        <is>
+          <t>Nighty</t>
+        </is>
+      </c>
+      <c r="E1034" t="inlineStr">
+        <is>
+          <t>Short Sleeves</t>
+        </is>
+      </c>
+      <c r="F1034" t="inlineStr">
+        <is>
+          <t>Square Neck</t>
+        </is>
+      </c>
+      <c r="G1034" t="inlineStr">
+        <is>
+          <t>SINGLE DRESS</t>
+        </is>
+      </c>
+      <c r="H1034" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="I1034" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="J1034" t="n">
+        <v>1</v>
+      </c>
+      <c r="K1034" t="inlineStr">
+        <is>
+          <t>Navy Blue</t>
+        </is>
+      </c>
+      <c r="L1034" t="inlineStr">
+        <is>
+          <t>XXL</t>
+        </is>
+      </c>
+      <c r="M1034" t="n">
+        <v>1</v>
+      </c>
+      <c r="N1034" t="inlineStr">
+        <is>
+          <t>DE26010N101313</t>
+        </is>
+      </c>
+      <c r="O1034" t="n">
+        <v>185</v>
+      </c>
+      <c r="P1034" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="Q1034">
+        <f>ROUND($O1034+10+($O1034*0.2)+(($O1034+10+($O1034*0.2))*$P1034)+(($O1034+10+($O1034*0.2)+(($O1034+10+($O1034*0.2))*$P1034))*0.05),0)</f>
+        <v/>
+      </c>
+      <c r="R1034" t="n">
+        <v>449</v>
+      </c>
+      <c r="S1034" t="n">
+        <v>449</v>
+      </c>
+      <c r="T1034" t="inlineStr">
+        <is>
+          <t>PDE26010N101313</t>
+        </is>
+      </c>
+    </row>
+    <row r="1035">
+      <c r="A1035" t="n">
+        <v>51</v>
+      </c>
+      <c r="B1035" t="inlineStr">
+        <is>
+          <t>Everyday</t>
+        </is>
+      </c>
+      <c r="C1035" t="inlineStr">
+        <is>
+          <t>DE26010R</t>
+        </is>
+      </c>
+      <c r="D1035" t="inlineStr">
+        <is>
+          <t>Nighty</t>
+        </is>
+      </c>
+      <c r="E1035" t="inlineStr">
+        <is>
+          <t>Short Sleeves</t>
+        </is>
+      </c>
+      <c r="F1035" t="inlineStr">
+        <is>
+          <t>Square Neck</t>
+        </is>
+      </c>
+      <c r="G1035" t="inlineStr">
+        <is>
+          <t>SINGLE DRESS</t>
+        </is>
+      </c>
+      <c r="H1035" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="I1035" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="J1035" t="n">
+        <v>1</v>
+      </c>
+      <c r="K1035" t="inlineStr">
+        <is>
+          <t>Red</t>
+        </is>
+      </c>
+      <c r="L1035" t="inlineStr">
+        <is>
+          <t>XXL</t>
+        </is>
+      </c>
+      <c r="M1035" t="n">
+        <v>1</v>
+      </c>
+      <c r="N1035" t="inlineStr">
+        <is>
+          <t>DE26010R101213</t>
+        </is>
+      </c>
+      <c r="O1035" t="n">
+        <v>185</v>
+      </c>
+      <c r="P1035" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="Q1035">
+        <f>ROUND($O1035+10+($O1035*0.2)+(($O1035+10+($O1035*0.2))*$P1035)+(($O1035+10+($O1035*0.2)+(($O1035+10+($O1035*0.2))*$P1035))*0.05),0)</f>
+        <v/>
+      </c>
+      <c r="R1035" t="n">
+        <v>449</v>
+      </c>
+      <c r="S1035" t="n">
+        <v>449</v>
+      </c>
+      <c r="T1035" t="inlineStr">
+        <is>
+          <t>PDE26010R101213</t>
+        </is>
+      </c>
+    </row>
+    <row r="1036">
+      <c r="A1036" t="n">
+        <v>62</v>
+      </c>
+      <c r="B1036" t="inlineStr">
+        <is>
+          <t>Everyday</t>
+        </is>
+      </c>
+      <c r="C1036" t="inlineStr">
+        <is>
+          <t>DE26_A47038</t>
+        </is>
+      </c>
+      <c r="D1036" t="inlineStr">
+        <is>
+          <t>Nighty</t>
+        </is>
+      </c>
+      <c r="E1036" t="inlineStr">
+        <is>
+          <t>Sleeveless</t>
+        </is>
+      </c>
+      <c r="F1036" t="inlineStr">
+        <is>
+          <t>Square Neck</t>
+        </is>
+      </c>
+      <c r="G1036" t="inlineStr">
+        <is>
+          <t>SINGLE DRESS</t>
+        </is>
+      </c>
+      <c r="H1036" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="I1036" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="J1036" t="n">
+        <v>1</v>
+      </c>
+      <c r="K1036" t="inlineStr">
+        <is>
+          <t>Teal</t>
+        </is>
+      </c>
+      <c r="L1036" t="inlineStr">
+        <is>
+          <t>XXL</t>
+        </is>
+      </c>
+      <c r="M1036" t="n">
+        <v>1</v>
+      </c>
+      <c r="N1036" t="inlineStr">
+        <is>
+          <t>DE26_A47038103313</t>
+        </is>
+      </c>
+      <c r="O1036" t="n">
+        <v>210</v>
+      </c>
+      <c r="P1036" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="Q1036">
+        <f>ROUND($O1036+10+($O1036*0.2)+(($O1036+10+($O1036*0.2))*$P1036)+(($O1036+10+($O1036*0.2)+(($O1036+10+($O1036*0.2))*$P1036))*0.05),0)</f>
+        <v/>
+      </c>
+      <c r="R1036" t="n">
+        <v>499</v>
+      </c>
+      <c r="S1036" t="n">
+        <v>499</v>
+      </c>
+      <c r="T1036" t="inlineStr">
+        <is>
+          <t>PDE26_A47038103313</t>
+        </is>
+      </c>
+    </row>
+    <row r="1037">
+      <c r="A1037" t="n">
+        <v>63</v>
+      </c>
+      <c r="B1037" t="inlineStr">
+        <is>
+          <t>Everyday</t>
+        </is>
+      </c>
+      <c r="C1037" t="inlineStr">
+        <is>
+          <t>TESTDEL_2EAD12</t>
+        </is>
+      </c>
+      <c r="D1037" t="inlineStr">
+        <is>
+          <t>Women</t>
+        </is>
+      </c>
+      <c r="E1037" t="inlineStr">
+        <is>
+          <t>Nightdress</t>
+        </is>
+      </c>
+      <c r="F1037" t="inlineStr">
+        <is>
+          <t>Maxi</t>
+        </is>
+      </c>
+      <c r="G1037" t="inlineStr">
+        <is>
+          <t>SINGLE DRESS</t>
+        </is>
+      </c>
+      <c r="H1037" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="I1037" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="J1037" t="n">
+        <v>1</v>
+      </c>
+      <c r="K1037" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="L1037" t="inlineStr">
+        <is>
+          <t>XXL</t>
+        </is>
+      </c>
+      <c r="M1037" t="n">
+        <v>1</v>
+      </c>
+      <c r="N1037" t="inlineStr">
+        <is>
+          <t>TESTDEL_2EAD12103813</t>
+        </is>
+      </c>
+      <c r="O1037" t="n">
+        <v>150</v>
+      </c>
+      <c r="P1037" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="Q1037">
+        <f>ROUND($O1037+10+($O1037*0.2)+(($O1037+10+($O1037*0.2))*$P1037)+(($O1037+10+($O1037*0.2)+(($O1037+10+($O1037*0.2))*$P1037))*0.05),0)</f>
+        <v/>
+      </c>
+      <c r="R1037" t="n">
+        <v>499</v>
+      </c>
+      <c r="S1037" t="n">
+        <v>499</v>
+      </c>
+      <c r="T1037" t="inlineStr">
+        <is>
+          <t>PTESTDEL_2EAD12103813</t>
+        </is>
+      </c>
+    </row>
+    <row r="1038">
+      <c r="A1038" t="n">
+        <v>63</v>
+      </c>
+      <c r="B1038" t="inlineStr">
+        <is>
+          <t>Everyday</t>
+        </is>
+      </c>
+      <c r="C1038" t="inlineStr">
+        <is>
+          <t>TESTIMG_130CE2</t>
+        </is>
+      </c>
+      <c r="D1038" t="inlineStr">
+        <is>
+          <t>Nighty</t>
+        </is>
+      </c>
+      <c r="E1038" t="inlineStr">
+        <is>
+          <t>Sleeveless</t>
+        </is>
+      </c>
+      <c r="F1038" t="inlineStr">
+        <is>
+          <t>Square Neck</t>
+        </is>
+      </c>
+      <c r="G1038" t="inlineStr">
+        <is>
+          <t>SINGLE DRESS</t>
+        </is>
+      </c>
+      <c r="H1038" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="I1038" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="J1038" t="n">
+        <v>1</v>
+      </c>
+      <c r="K1038" t="inlineStr">
+        <is>
+          <t>Blue</t>
+        </is>
+      </c>
+      <c r="L1038" t="inlineStr">
+        <is>
+          <t>XXL</t>
+        </is>
+      </c>
+      <c r="M1038" t="n">
+        <v>1</v>
+      </c>
+      <c r="N1038" t="inlineStr">
+        <is>
+          <t>TESTIMG_130CE2103613</t>
+        </is>
+      </c>
+      <c r="O1038" t="n">
+        <v>185</v>
+      </c>
+      <c r="P1038" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="Q1038">
+        <f>ROUND($O1038+10+($O1038*0.2)+(($O1038+10+($O1038*0.2))*$P1038)+(($O1038+10+($O1038*0.2)+(($O1038+10+($O1038*0.2))*$P1038))*0.05),0)</f>
+        <v/>
+      </c>
+      <c r="R1038" t="n">
+        <v>499</v>
+      </c>
+      <c r="S1038" t="n">
+        <v>499</v>
+      </c>
+      <c r="T1038" t="inlineStr">
+        <is>
+          <t>PTESTIMG_130CE2103613</t>
+        </is>
+      </c>
+    </row>
+    <row r="1039">
+      <c r="A1039" t="n">
+        <v>64</v>
+      </c>
+      <c r="B1039" t="inlineStr">
+        <is>
+          <t>Everyday</t>
+        </is>
+      </c>
+      <c r="C1039" t="inlineStr">
+        <is>
+          <t>DE26_B79C0C</t>
+        </is>
+      </c>
+      <c r="D1039" t="inlineStr">
+        <is>
+          <t>Nighty</t>
+        </is>
+      </c>
+      <c r="E1039" t="inlineStr">
+        <is>
+          <t>Sleeveless</t>
+        </is>
+      </c>
+      <c r="F1039" t="inlineStr">
+        <is>
+          <t>Square Neck</t>
+        </is>
+      </c>
+      <c r="G1039" t="inlineStr">
+        <is>
+          <t>SINGLE DRESS</t>
+        </is>
+      </c>
+      <c r="H1039" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="I1039" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="J1039" t="n">
+        <v>1</v>
+      </c>
+      <c r="K1039" t="inlineStr">
+        <is>
+          <t>Teal</t>
+        </is>
+      </c>
+      <c r="L1039" t="inlineStr">
+        <is>
+          <t>XXL</t>
+        </is>
+      </c>
+      <c r="M1039" t="n">
+        <v>1</v>
+      </c>
+      <c r="N1039" t="inlineStr">
+        <is>
+          <t>DE26_B79C0C103313</t>
+        </is>
+      </c>
+      <c r="O1039" t="n">
+        <v>210</v>
+      </c>
+      <c r="P1039" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="Q1039">
+        <f>ROUND($O1039+10+($O1039*0.2)+(($O1039+10+($O1039*0.2))*$P1039)+(($O1039+10+($O1039*0.2)+(($O1039+10+($O1039*0.2))*$P1039))*0.05),0)</f>
+        <v/>
+      </c>
+      <c r="R1039" t="n">
+        <v>499</v>
+      </c>
+      <c r="S1039" t="n">
+        <v>499</v>
+      </c>
+      <c r="T1039" t="inlineStr">
+        <is>
+          <t>PDE26_B79C0C103313</t>
+        </is>
+      </c>
+    </row>
+    <row r="1040">
+      <c r="A1040" t="n">
+        <v>65</v>
+      </c>
+      <c r="B1040" t="inlineStr">
+        <is>
+          <t>Everyday</t>
+        </is>
+      </c>
+      <c r="C1040" t="inlineStr">
+        <is>
+          <t>TESTDEL_B61EA2</t>
+        </is>
+      </c>
+      <c r="D1040" t="inlineStr">
+        <is>
+          <t>Women</t>
+        </is>
+      </c>
+      <c r="E1040" t="inlineStr">
+        <is>
+          <t>Nightdress</t>
+        </is>
+      </c>
+      <c r="F1040" t="inlineStr">
+        <is>
+          <t>Maxi</t>
+        </is>
+      </c>
+      <c r="G1040" t="inlineStr">
+        <is>
+          <t>SINGLE DRESS</t>
+        </is>
+      </c>
+      <c r="H1040" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="I1040" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="J1040" t="n">
+        <v>1</v>
+      </c>
+      <c r="K1040" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="L1040" t="inlineStr">
+        <is>
+          <t>XXL</t>
+        </is>
+      </c>
+      <c r="M1040" t="n">
+        <v>1</v>
+      </c>
+      <c r="N1040" t="inlineStr">
+        <is>
+          <t>TESTDEL_B61EA2103813</t>
+        </is>
+      </c>
+      <c r="O1040" t="n">
+        <v>150</v>
+      </c>
+      <c r="P1040" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="Q1040">
+        <f>ROUND($O1040+10+($O1040*0.2)+(($O1040+10+($O1040*0.2))*$P1040)+(($O1040+10+($O1040*0.2)+(($O1040+10+($O1040*0.2))*$P1040))*0.05),0)</f>
+        <v/>
+      </c>
+      <c r="R1040" t="n">
+        <v>499</v>
+      </c>
+      <c r="S1040" t="n">
+        <v>499</v>
+      </c>
+      <c r="T1040" t="inlineStr">
+        <is>
+          <t>PTESTDEL_B61EA2103813</t>
+        </is>
+      </c>
+    </row>
+    <row r="1041">
+      <c r="A1041" t="n">
+        <v>65</v>
+      </c>
+      <c r="B1041" t="inlineStr">
+        <is>
+          <t>Everyday</t>
+        </is>
+      </c>
+      <c r="C1041" t="inlineStr">
+        <is>
+          <t>TESTIMG_297FAE</t>
+        </is>
+      </c>
+      <c r="D1041" t="inlineStr">
+        <is>
+          <t>Nighty</t>
+        </is>
+      </c>
+      <c r="E1041" t="inlineStr">
+        <is>
+          <t>Sleeveless</t>
+        </is>
+      </c>
+      <c r="F1041" t="inlineStr">
+        <is>
+          <t>Square Neck</t>
+        </is>
+      </c>
+      <c r="G1041" t="inlineStr">
+        <is>
+          <t>SINGLE DRESS</t>
+        </is>
+      </c>
+      <c r="H1041" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="I1041" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="J1041" t="n">
+        <v>1</v>
+      </c>
+      <c r="K1041" t="inlineStr">
+        <is>
+          <t>Blue</t>
+        </is>
+      </c>
+      <c r="L1041" t="inlineStr">
+        <is>
+          <t>XXL</t>
+        </is>
+      </c>
+      <c r="M1041" t="n">
+        <v>1</v>
+      </c>
+      <c r="N1041" t="inlineStr">
+        <is>
+          <t>TESTIMG_297FAE103613</t>
+        </is>
+      </c>
+      <c r="O1041" t="n">
+        <v>185</v>
+      </c>
+      <c r="P1041" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="Q1041">
+        <f>ROUND($O1041+10+($O1041*0.2)+(($O1041+10+($O1041*0.2))*$P1041)+(($O1041+10+($O1041*0.2)+(($O1041+10+($O1041*0.2))*$P1041))*0.05),0)</f>
+        <v/>
+      </c>
+      <c r="R1041" t="n">
+        <v>499</v>
+      </c>
+      <c r="S1041" t="n">
+        <v>499</v>
+      </c>
+      <c r="T1041" t="inlineStr">
+        <is>
+          <t>PTESTIMG_297FAE103613</t>
+        </is>
+      </c>
+    </row>
+    <row r="1042">
+      <c r="A1042" t="n">
+        <v>52</v>
+      </c>
+      <c r="B1042" t="inlineStr">
+        <is>
+          <t>Everyday</t>
+        </is>
+      </c>
+      <c r="C1042" t="inlineStr">
+        <is>
+          <t>DE26012K</t>
+        </is>
+      </c>
+      <c r="D1042" t="inlineStr">
+        <is>
+          <t>Nighty</t>
+        </is>
+      </c>
+      <c r="E1042" t="inlineStr">
+        <is>
+          <t>Sleeveless</t>
+        </is>
+      </c>
+      <c r="F1042" t="inlineStr">
+        <is>
+          <t>Stylised</t>
+        </is>
+      </c>
+      <c r="G1042" t="inlineStr">
+        <is>
+          <t>SINGLE DRESS</t>
+        </is>
+      </c>
+      <c r="H1042" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="I1042" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="J1042" t="n">
+        <v>1</v>
+      </c>
+      <c r="K1042" t="inlineStr">
+        <is>
+          <t>Black</t>
+        </is>
+      </c>
+      <c r="L1042" t="inlineStr">
+        <is>
+          <t>XXL</t>
+        </is>
+      </c>
+      <c r="M1042" t="n">
+        <v>1</v>
+      </c>
+      <c r="N1042" t="inlineStr">
+        <is>
+          <t>DE26012K103313</t>
+        </is>
+      </c>
+      <c r="O1042" t="n">
+        <v>225</v>
+      </c>
+      <c r="P1042" t="n">
+        <v>0.217</v>
+      </c>
+      <c r="Q1042">
+        <f>ROUND($O1042+10+($O1042*0.2)+(($O1042+10+($O1042*0.2))*$P1042)+(($O1042+10+($O1042*0.2)+(($O1042+10+($O1042*0.2))*$P1042))*0.05),0)</f>
+        <v/>
+      </c>
+      <c r="R1042" t="n">
+        <v>599</v>
+      </c>
+      <c r="S1042" t="n">
+        <v>599</v>
+      </c>
+      <c r="T1042" t="inlineStr">
+        <is>
+          <t>PDE26012K103313</t>
+        </is>
+      </c>
+    </row>
+    <row r="1043">
+      <c r="A1043" t="n">
+        <v>53</v>
+      </c>
+      <c r="B1043" t="inlineStr">
+        <is>
+          <t>Everyday</t>
+        </is>
+      </c>
+      <c r="C1043" t="inlineStr">
+        <is>
+          <t>DE26012B</t>
+        </is>
+      </c>
+      <c r="D1043" t="inlineStr">
+        <is>
+          <t>Nighty</t>
+        </is>
+      </c>
+      <c r="E1043" t="inlineStr">
+        <is>
+          <t>Sleeveless</t>
+        </is>
+      </c>
+      <c r="F1043" t="inlineStr">
+        <is>
+          <t>Stylised</t>
+        </is>
+      </c>
+      <c r="G1043" t="inlineStr">
+        <is>
+          <t>SINGLE DRESS</t>
+        </is>
+      </c>
+      <c r="H1043" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="I1043" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="J1043" t="n">
+        <v>1</v>
+      </c>
+      <c r="K1043" t="inlineStr">
+        <is>
+          <t>Blue</t>
+        </is>
+      </c>
+      <c r="L1043" t="inlineStr">
+        <is>
+          <t>XXL</t>
+        </is>
+      </c>
+      <c r="M1043" t="n">
+        <v>1</v>
+      </c>
+      <c r="N1043" t="inlineStr">
+        <is>
+          <t>DE26012B103613</t>
+        </is>
+      </c>
+      <c r="O1043" t="n">
+        <v>225</v>
+      </c>
+      <c r="P1043" t="n">
+        <v>0.206</v>
+      </c>
+      <c r="Q1043">
+        <f>ROUND($O1043+10+($O1043*0.2)+(($O1043+10+($O1043*0.2))*$P1043)+(($O1043+10+($O1043*0.2)+(($O1043+10+($O1043*0.2))*$P1043))*0.05),0)</f>
+        <v/>
+      </c>
+      <c r="R1043" t="n">
+        <v>599</v>
+      </c>
+      <c r="S1043" t="n">
+        <v>599</v>
+      </c>
+      <c r="T1043" t="inlineStr">
+        <is>
+          <t>PDE26012B103613</t>
+        </is>
+      </c>
+    </row>
+    <row r="1044">
+      <c r="A1044" t="n">
+        <v>66</v>
+      </c>
+      <c r="B1044" t="inlineStr">
+        <is>
+          <t>Everyday</t>
+        </is>
+      </c>
+      <c r="C1044" t="inlineStr">
+        <is>
+          <t>DE26_FF9631</t>
+        </is>
+      </c>
+      <c r="D1044" t="inlineStr">
+        <is>
+          <t>Nighty</t>
+        </is>
+      </c>
+      <c r="E1044" t="inlineStr">
+        <is>
+          <t>Sleeveless</t>
+        </is>
+      </c>
+      <c r="F1044" t="inlineStr">
+        <is>
+          <t>Square Neck</t>
+        </is>
+      </c>
+      <c r="G1044" t="inlineStr">
+        <is>
+          <t>SINGLE DRESS</t>
+        </is>
+      </c>
+      <c r="H1044" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="I1044" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="J1044" t="n">
+        <v>1</v>
+      </c>
+      <c r="K1044" t="inlineStr">
+        <is>
+          <t>Teal</t>
+        </is>
+      </c>
+      <c r="L1044" t="inlineStr">
+        <is>
+          <t>XXL</t>
+        </is>
+      </c>
+      <c r="M1044" t="n">
+        <v>1</v>
+      </c>
+      <c r="N1044" t="inlineStr">
+        <is>
+          <t>DE26_FF9631103313</t>
+        </is>
+      </c>
+      <c r="O1044" t="n">
+        <v>210</v>
+      </c>
+      <c r="P1044" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="Q1044">
+        <f>ROUND($O1044+10+($O1044*0.2)+(($O1044+10+($O1044*0.2))*$P1044)+(($O1044+10+($O1044*0.2)+(($O1044+10+($O1044*0.2))*$P1044))*0.05),0)</f>
+        <v/>
+      </c>
+      <c r="R1044" t="n">
+        <v>499</v>
+      </c>
+      <c r="S1044" t="n">
+        <v>499</v>
+      </c>
+      <c r="T1044" t="inlineStr">
+        <is>
+          <t>PDE26_FF9631103313</t>
+        </is>
+      </c>
+    </row>
+    <row r="1045">
+      <c r="A1045" t="n">
+        <v>67</v>
+      </c>
+      <c r="B1045" t="inlineStr">
+        <is>
+          <t>Everyday</t>
+        </is>
+      </c>
+      <c r="C1045" t="inlineStr">
+        <is>
+          <t>TESTDEL_D318F3</t>
+        </is>
+      </c>
+      <c r="D1045" t="inlineStr">
+        <is>
+          <t>Women</t>
+        </is>
+      </c>
+      <c r="E1045" t="inlineStr">
+        <is>
+          <t>Nightdress</t>
+        </is>
+      </c>
+      <c r="F1045" t="inlineStr">
+        <is>
+          <t>Maxi</t>
+        </is>
+      </c>
+      <c r="G1045" t="inlineStr">
+        <is>
+          <t>SINGLE DRESS</t>
+        </is>
+      </c>
+      <c r="H1045" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="I1045" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="J1045" t="n">
+        <v>1</v>
+      </c>
+      <c r="K1045" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="L1045" t="inlineStr">
+        <is>
+          <t>XXL</t>
+        </is>
+      </c>
+      <c r="M1045" t="n">
+        <v>1</v>
+      </c>
+      <c r="N1045" t="inlineStr">
+        <is>
+          <t>TESTDEL_D318F3103813</t>
+        </is>
+      </c>
+      <c r="O1045" t="n">
+        <v>150</v>
+      </c>
+      <c r="P1045" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="Q1045">
+        <f>ROUND($O1045+10+($O1045*0.2)+(($O1045+10+($O1045*0.2))*$P1045)+(($O1045+10+($O1045*0.2)+(($O1045+10+($O1045*0.2))*$P1045))*0.05),0)</f>
+        <v/>
+      </c>
+      <c r="R1045" t="n">
+        <v>499</v>
+      </c>
+      <c r="S1045" t="n">
+        <v>499</v>
+      </c>
+      <c r="T1045" t="inlineStr">
+        <is>
+          <t>PTESTDEL_D318F3103813</t>
+        </is>
+      </c>
+    </row>
+    <row r="1046">
+      <c r="A1046" t="n">
+        <v>67</v>
+      </c>
+      <c r="B1046" t="inlineStr">
+        <is>
+          <t>Everyday</t>
+        </is>
+      </c>
+      <c r="C1046" t="inlineStr">
+        <is>
+          <t>TESTIMG_3D9312</t>
+        </is>
+      </c>
+      <c r="D1046" t="inlineStr">
+        <is>
+          <t>Nighty</t>
+        </is>
+      </c>
+      <c r="E1046" t="inlineStr">
+        <is>
+          <t>Sleeveless</t>
+        </is>
+      </c>
+      <c r="F1046" t="inlineStr">
+        <is>
+          <t>Square Neck</t>
+        </is>
+      </c>
+      <c r="G1046" t="inlineStr">
+        <is>
+          <t>SINGLE DRESS</t>
+        </is>
+      </c>
+      <c r="H1046" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="I1046" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="J1046" t="n">
+        <v>1</v>
+      </c>
+      <c r="K1046" t="inlineStr">
+        <is>
+          <t>Blue</t>
+        </is>
+      </c>
+      <c r="L1046" t="inlineStr">
+        <is>
+          <t>XXL</t>
+        </is>
+      </c>
+      <c r="M1046" t="n">
+        <v>1</v>
+      </c>
+      <c r="N1046" t="inlineStr">
+        <is>
+          <t>TESTIMG_3D9312103613</t>
+        </is>
+      </c>
+      <c r="O1046" t="n">
+        <v>185</v>
+      </c>
+      <c r="P1046" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="Q1046">
+        <f>ROUND($O1046+10+($O1046*0.2)+(($O1046+10+($O1046*0.2))*$P1046)+(($O1046+10+($O1046*0.2)+(($O1046+10+($O1046*0.2))*$P1046))*0.05),0)</f>
+        <v/>
+      </c>
+      <c r="R1046" t="n">
+        <v>499</v>
+      </c>
+      <c r="S1046" t="n">
+        <v>499</v>
+      </c>
+      <c r="T1046" t="inlineStr">
+        <is>
+          <t>PTESTIMG_3D9312103613</t>
+        </is>
+      </c>
+    </row>
+    <row r="1047">
+      <c r="A1047" t="n">
+        <v>68</v>
+      </c>
+      <c r="B1047" t="inlineStr">
+        <is>
+          <t>Everyday</t>
+        </is>
+      </c>
+      <c r="C1047" t="inlineStr">
+        <is>
+          <t>DE26_D5F52E</t>
+        </is>
+      </c>
+      <c r="D1047" t="inlineStr">
+        <is>
+          <t>Nighty</t>
+        </is>
+      </c>
+      <c r="E1047" t="inlineStr">
+        <is>
+          <t>Sleeveless</t>
+        </is>
+      </c>
+      <c r="F1047" t="inlineStr">
+        <is>
+          <t>Square Neck</t>
+        </is>
+      </c>
+      <c r="G1047" t="inlineStr">
+        <is>
+          <t>SINGLE DRESS</t>
+        </is>
+      </c>
+      <c r="H1047" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="I1047" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="J1047" t="n">
+        <v>1</v>
+      </c>
+      <c r="K1047" t="inlineStr">
+        <is>
+          <t>Teal</t>
+        </is>
+      </c>
+      <c r="L1047" t="inlineStr">
+        <is>
+          <t>XXL</t>
+        </is>
+      </c>
+      <c r="M1047" t="n">
+        <v>1</v>
+      </c>
+      <c r="N1047" t="inlineStr">
+        <is>
+          <t>DE26_D5F52E103313</t>
+        </is>
+      </c>
+      <c r="O1047" t="n">
+        <v>210</v>
+      </c>
+      <c r="P1047" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="Q1047">
+        <f>ROUND($O1047+10+($O1047*0.2)+(($O1047+10+($O1047*0.2))*$P1047)+(($O1047+10+($O1047*0.2)+(($O1047+10+($O1047*0.2))*$P1047))*0.05),0)</f>
+        <v/>
+      </c>
+      <c r="R1047" t="n">
+        <v>499</v>
+      </c>
+      <c r="S1047" t="n">
+        <v>499</v>
+      </c>
+      <c r="T1047" t="inlineStr">
+        <is>
+          <t>PDE26_D5F52E103313</t>
+        </is>
+      </c>
+    </row>
+    <row r="1048">
+      <c r="A1048" t="n">
+        <v>69</v>
+      </c>
+      <c r="B1048" t="inlineStr">
+        <is>
+          <t>Everyday</t>
+        </is>
+      </c>
+      <c r="C1048" t="inlineStr">
+        <is>
+          <t>TESTDEL_09285F</t>
+        </is>
+      </c>
+      <c r="D1048" t="inlineStr">
+        <is>
+          <t>Women</t>
+        </is>
+      </c>
+      <c r="E1048" t="inlineStr">
+        <is>
+          <t>Nightdress</t>
+        </is>
+      </c>
+      <c r="F1048" t="inlineStr">
+        <is>
+          <t>Maxi</t>
+        </is>
+      </c>
+      <c r="G1048" t="inlineStr">
+        <is>
+          <t>SINGLE DRESS</t>
+        </is>
+      </c>
+      <c r="H1048" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="I1048" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="J1048" t="n">
+        <v>1</v>
+      </c>
+      <c r="K1048" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="L1048" t="inlineStr">
+        <is>
+          <t>XXL</t>
+        </is>
+      </c>
+      <c r="M1048" t="n">
+        <v>1</v>
+      </c>
+      <c r="N1048" t="inlineStr">
+        <is>
+          <t>TESTDEL_09285F103813</t>
+        </is>
+      </c>
+      <c r="O1048" t="n">
+        <v>150</v>
+      </c>
+      <c r="P1048" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="Q1048">
+        <f>ROUND($O1048+10+($O1048*0.2)+(($O1048+10+($O1048*0.2))*$P1048)+(($O1048+10+($O1048*0.2)+(($O1048+10+($O1048*0.2))*$P1048))*0.05),0)</f>
+        <v/>
+      </c>
+      <c r="R1048" t="n">
+        <v>499</v>
+      </c>
+      <c r="S1048" t="n">
+        <v>499</v>
+      </c>
+      <c r="T1048" t="inlineStr">
+        <is>
+          <t>PTESTDEL_09285F103813</t>
+        </is>
+      </c>
+    </row>
+    <row r="1049">
+      <c r="A1049" t="n">
+        <v>69</v>
+      </c>
+      <c r="B1049" t="inlineStr">
+        <is>
+          <t>Everyday</t>
+        </is>
+      </c>
+      <c r="C1049" t="inlineStr">
+        <is>
+          <t>TESTIMG_6855A1</t>
+        </is>
+      </c>
+      <c r="D1049" t="inlineStr">
+        <is>
+          <t>Nighty</t>
+        </is>
+      </c>
+      <c r="E1049" t="inlineStr">
+        <is>
+          <t>Sleeveless</t>
+        </is>
+      </c>
+      <c r="F1049" t="inlineStr">
+        <is>
+          <t>Square Neck</t>
+        </is>
+      </c>
+      <c r="G1049" t="inlineStr">
+        <is>
+          <t>SINGLE DRESS</t>
+        </is>
+      </c>
+      <c r="H1049" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="I1049" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="J1049" t="n">
+        <v>1</v>
+      </c>
+      <c r="K1049" t="inlineStr">
+        <is>
+          <t>Blue</t>
+        </is>
+      </c>
+      <c r="L1049" t="inlineStr">
+        <is>
+          <t>XXL</t>
+        </is>
+      </c>
+      <c r="M1049" t="n">
+        <v>1</v>
+      </c>
+      <c r="N1049" t="inlineStr">
+        <is>
+          <t>TESTIMG_6855A1103613</t>
+        </is>
+      </c>
+      <c r="O1049" t="n">
+        <v>185</v>
+      </c>
+      <c r="P1049" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="Q1049">
+        <f>ROUND($O1049+10+($O1049*0.2)+(($O1049+10+($O1049*0.2))*$P1049)+(($O1049+10+($O1049*0.2)+(($O1049+10+($O1049*0.2))*$P1049))*0.05),0)</f>
+        <v/>
+      </c>
+      <c r="R1049" t="n">
+        <v>499</v>
+      </c>
+      <c r="S1049" t="n">
+        <v>499</v>
+      </c>
+      <c r="T1049" t="inlineStr">
+        <is>
+          <t>PTESTIMG_6855A1103613</t>
+        </is>
+      </c>
+    </row>
+    <row r="1050">
+      <c r="A1050" t="n">
+        <v>70</v>
+      </c>
+      <c r="B1050" t="inlineStr">
+        <is>
+          <t>Everyday</t>
+        </is>
+      </c>
+      <c r="C1050" t="inlineStr">
+        <is>
+          <t>DE26_C7F704</t>
+        </is>
+      </c>
+      <c r="D1050" t="inlineStr">
+        <is>
+          <t>Nighty</t>
+        </is>
+      </c>
+      <c r="E1050" t="inlineStr">
+        <is>
+          <t>Sleeveless</t>
+        </is>
+      </c>
+      <c r="F1050" t="inlineStr">
+        <is>
+          <t>Square Neck</t>
+        </is>
+      </c>
+      <c r="G1050" t="inlineStr">
+        <is>
+          <t>SINGLE DRESS</t>
+        </is>
+      </c>
+      <c r="H1050" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="I1050" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="J1050" t="n">
+        <v>1</v>
+      </c>
+      <c r="K1050" t="inlineStr">
+        <is>
+          <t>Teal</t>
+        </is>
+      </c>
+      <c r="L1050" t="inlineStr">
+        <is>
+          <t>XXL</t>
+        </is>
+      </c>
+      <c r="M1050" t="n">
+        <v>1</v>
+      </c>
+      <c r="N1050" t="inlineStr">
+        <is>
+          <t>DE26_C7F704103313</t>
+        </is>
+      </c>
+      <c r="O1050" t="n">
+        <v>210</v>
+      </c>
+      <c r="P1050" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="Q1050">
+        <f>ROUND($O1050+10+($O1050*0.2)+(($O1050+10+($O1050*0.2))*$P1050)+(($O1050+10+($O1050*0.2)+(($O1050+10+($O1050*0.2))*$P1050))*0.05),0)</f>
+        <v/>
+      </c>
+      <c r="R1050" t="n">
+        <v>499</v>
+      </c>
+      <c r="S1050" t="n">
+        <v>499</v>
+      </c>
+      <c r="T1050" t="inlineStr">
+        <is>
+          <t>PDE26_C7F704103313</t>
+        </is>
+      </c>
+    </row>
+    <row r="1051">
+      <c r="A1051" t="n">
+        <v>71</v>
+      </c>
+      <c r="B1051" t="inlineStr">
+        <is>
+          <t>Everyday</t>
+        </is>
+      </c>
+      <c r="C1051" t="inlineStr">
+        <is>
+          <t>TESTDEL_85BE32</t>
+        </is>
+      </c>
+      <c r="D1051" t="inlineStr">
+        <is>
+          <t>Women</t>
+        </is>
+      </c>
+      <c r="E1051" t="inlineStr">
+        <is>
+          <t>Nightdress</t>
+        </is>
+      </c>
+      <c r="F1051" t="inlineStr">
+        <is>
+          <t>Maxi</t>
+        </is>
+      </c>
+      <c r="G1051" t="inlineStr">
+        <is>
+          <t>SINGLE DRESS</t>
+        </is>
+      </c>
+      <c r="H1051" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="I1051" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="J1051" t="n">
+        <v>1</v>
+      </c>
+      <c r="K1051" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="L1051" t="inlineStr">
+        <is>
+          <t>XXL</t>
+        </is>
+      </c>
+      <c r="M1051" t="n">
+        <v>1</v>
+      </c>
+      <c r="N1051" t="inlineStr">
+        <is>
+          <t>TESTDEL_85BE32103813</t>
+        </is>
+      </c>
+      <c r="O1051" t="n">
+        <v>150</v>
+      </c>
+      <c r="P1051" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="Q1051">
+        <f>ROUND($O1051+10+($O1051*0.2)+(($O1051+10+($O1051*0.2))*$P1051)+(($O1051+10+($O1051*0.2)+(($O1051+10+($O1051*0.2))*$P1051))*0.05),0)</f>
+        <v/>
+      </c>
+      <c r="R1051" t="n">
+        <v>499</v>
+      </c>
+      <c r="S1051" t="n">
+        <v>499</v>
+      </c>
+      <c r="T1051" t="inlineStr">
+        <is>
+          <t>PTESTDEL_85BE32103813</t>
+        </is>
+      </c>
+    </row>
+    <row r="1052">
+      <c r="A1052" t="n">
+        <v>71</v>
+      </c>
+      <c r="B1052" t="inlineStr">
+        <is>
+          <t>Everyday</t>
+        </is>
+      </c>
+      <c r="C1052" t="inlineStr">
+        <is>
+          <t>TESTIMG_47F849</t>
+        </is>
+      </c>
+      <c r="D1052" t="inlineStr">
+        <is>
+          <t>Nighty</t>
+        </is>
+      </c>
+      <c r="E1052" t="inlineStr">
+        <is>
+          <t>Sleeveless</t>
+        </is>
+      </c>
+      <c r="F1052" t="inlineStr">
+        <is>
+          <t>Square Neck</t>
+        </is>
+      </c>
+      <c r="G1052" t="inlineStr">
+        <is>
+          <t>SINGLE DRESS</t>
+        </is>
+      </c>
+      <c r="H1052" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="I1052" t="inlineStr">
+        <is>
+          <t>Woven</t>
+        </is>
+      </c>
+      <c r="J1052" t="n">
+        <v>1</v>
+      </c>
+      <c r="K1052" t="inlineStr">
+        <is>
+          <t>Blue</t>
+        </is>
+      </c>
+      <c r="L1052" t="inlineStr">
+        <is>
+          <t>XXL</t>
+        </is>
+      </c>
+      <c r="M1052" t="n">
+        <v>1</v>
+      </c>
+      <c r="N1052" t="inlineStr">
+        <is>
+          <t>TESTIMG_47F849103613</t>
+        </is>
+      </c>
+      <c r="O1052" t="n">
+        <v>185</v>
+      </c>
+      <c r="P1052" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="Q1052">
+        <f>ROUND($O1052+10+($O1052*0.2)+(($O1052+10+($O1052*0.2))*$P1052)+(($O1052+10+($O1052*0.2)+(($O1052+10+($O1052*0.2))*$P1052))*0.05),0)</f>
+        <v/>
+      </c>
+      <c r="R1052" t="n">
+        <v>499</v>
+      </c>
+      <c r="S1052" t="n">
+        <v>499</v>
+      </c>
+      <c r="T1052" t="inlineStr">
+        <is>
+          <t>PTESTIMG_47F849103613</t>
         </is>
       </c>
     </row>

</xml_diff>